<commit_message>
EU layout: drop unused detail fields 18-24; keep row actions on one line
- TJXEWMS_PreticketLayout.xlsx: removed Detail lookup_id 18-24 (frdesc,
  engnoun, frnoun, item, fact1-3) via targeted XML row-delete so the
  remaining fields' formula sample values are preserved; recompiled JSON
  (Lane now 17 fields, skipped=0, byte-exact round-trip intact)
- styles.css: .del-cell white-space:nowrap so row ↑↓＋✕ buttons don't stack
  vertically when the table is wide (scroll instead of squeeze)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/OkFileDefinitions/TJXEWMS_PreticketLayout.xlsx
+++ b/data/OkFileDefinitions/TJXEWMS_PreticketLayout.xlsx
@@ -6288,9 +6288,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:ns3="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac">
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr defaultRowHeight="12" ns2:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" bestFit="1" customWidth="1"/>
@@ -6305,12 +6305,12 @@
     <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ns2:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ns2:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -6342,7 +6342,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ns2:dyDescent="0.2">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -6375,7 +6375,7 @@
         <v>001</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ns2:dyDescent="0.2">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -6408,7 +6408,7 @@
         <v>001</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ns2:dyDescent="0.2">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -6441,7 +6441,7 @@
         <v>3521</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ns2:dyDescent="0.2">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -6474,7 +6474,7 @@
         <v>750440</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ns2:dyDescent="0.2">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -6507,7 +6507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ns2:dyDescent="0.2">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -6540,7 +6540,7 @@
         <v xml:space="preserve">XL    </v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ns2:dyDescent="0.2">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -6573,7 +6573,7 @@
         <v>N</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" ns2:dyDescent="0.2">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -6606,7 +6606,7 @@
         <v xml:space="preserve">01        </v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ns2:dyDescent="0.2">
       <c r="A13" s="2">
         <v>9</v>
       </c>
@@ -6639,7 +6639,7 @@
         <v xml:space="preserve">          </v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ns2:dyDescent="0.2">
       <c r="A14" s="2">
         <v>10</v>
       </c>
@@ -6672,7 +6672,7 @@
         <v>003500</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ns2:dyDescent="0.2">
       <c r="A15" s="2">
         <v>11</v>
       </c>
@@ -6705,7 +6705,7 @@
         <v>N</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" ns2:dyDescent="0.2">
       <c r="A16" s="2">
         <v>12</v>
       </c>
@@ -6738,7 +6738,7 @@
         <v>999998</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" ns2:dyDescent="0.2">
       <c r="A17" s="2">
         <v>13</v>
       </c>
@@ -6771,7 +6771,7 @@
         <v>00003</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ns2:dyDescent="0.2">
       <c r="A18" s="2">
         <v>14</v>
       </c>
@@ -6804,7 +6804,7 @@
         <v>000000000</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" ns2:dyDescent="0.2">
       <c r="A19" s="2">
         <v>15</v>
       </c>
@@ -6837,7 +6837,7 @@
         <v>000</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" ns2:dyDescent="0.2">
       <c r="A20" s="2">
         <v>16</v>
       </c>
@@ -6870,7 +6870,7 @@
         <v>0000</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ns2:dyDescent="0.2">
       <c r="A21" s="2">
         <v>17</v>
       </c>
@@ -6903,240 +6903,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" s="2">
-        <v>18</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E22" s="2">
-        <v>20</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J22" s="5" t="str">
-        <f>IF(E22="","",MID($A$1, SUM($E$5:E22)-E22+1, E22))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" s="2">
-        <v>19</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E23" s="2">
-        <v>3</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J23" s="5" t="str">
-        <f>IF(E23="","",MID($A$1, SUM($E$5:E23)-E23+1, E23))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="2">
-        <v>20</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E24" s="2">
-        <v>3</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J24" s="5" t="str">
-        <f>IF(E24="","",MID($A$1, SUM($E$5:E24)-E24+1, E24))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" s="2">
-        <v>21</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E25" s="2">
-        <v>20</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J25" s="5" t="str">
-        <f>IF(E25="","",MID($A$1, SUM($E$5:E25)-E25+1, E25))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" s="2">
-        <v>22</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E26" s="2">
-        <v>20</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J26" s="5" t="str">
-        <f>IF(E26="","",MID($A$1, SUM($E$5:E26)-E26+1, E26))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="2">
-        <v>23</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E27" s="2">
-        <v>20</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J27" s="5" t="str">
-        <f>IF(E27="","",MID($A$1, SUM($E$5:E27)-E27+1, E27))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" s="2">
-        <v>24</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E28" s="2">
-        <v>20</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J28" s="5" t="str">
-        <f>IF(E28="","",MID($A$1, SUM($E$5:E28)-E28+1, E28))</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" ns3:id="rId1"/>
+  <legacyDrawing ns3:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
EU rename: lowercase xlsx tokens, EUPreticket preset, configurable region token
Lowercased the two capitalized field names in TJXEWMS_PreticketLayout.xlsx
(Indicator->indicator, Zone->zone) via a targeted shared-string XML edit so
the compiler no longer emits case-confusing tokens; cached formula values and
byte-exact round-trip preserved. Added the missing EU detail fields
(page/line/size/qty/ladder) to the rename palette and a new "EUPreticket
naming convension" preset.

New configurable `region` derived rename token: config/regions.yaml maps each
region to its zones (Reg1=01/03/05/33, Reg2=02/04/06/07/08/10); Config loads +
inverts it to zone->region and exposes Config.region(zone) (blank for
unmapped/non-EU). Wired into the rename token resolver + derived allowlist.

+1 config test, updated 2 EU field-name assertions (88 passing).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/OkFileDefinitions/TJXEWMS_PreticketLayout.xlsx
+++ b/data/OkFileDefinitions/TJXEWMS_PreticketLayout.xlsx
@@ -289,7 +289,7 @@
     <t xml:space="preserve">fact3                    </t>
   </si>
   <si>
-    <t>Indicator</t>
+    <t>indicator</t>
   </si>
   <si>
     <t>field001</t>
@@ -334,7 +334,7 @@
     <t>field014</t>
   </si>
   <si>
-    <t>Zone</t>
+    <t>zone</t>
   </si>
   <si>
     <t>P05A10021888 8720240710352102001001000126000000339810</t>

</xml_diff>